<commit_message>
update case of net primary productivity study
</commit_message>
<xml_diff>
--- a/Case of net primary productivity study/Case of net primary productivity study.xlsx
+++ b/Case of net primary productivity study/Case of net primary productivity study.xlsx
@@ -391,10 +391,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.6088477366255144</v>
+        <v>0.2181795918367347</v>
       </c>
       <c r="D2">
-        <v>8.929334696363851E-05</v>
+        <v>4.990672434241546E-48</v>
       </c>
     </row>
     <row r="3">
@@ -409,10 +409,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.5383539094650206</v>
+        <v>0.1876816326530612</v>
       </c>
       <c r="D3">
-        <v>0.1686403908193261</v>
+        <v>7.390330900445726E-67</v>
       </c>
     </row>
     <row r="4">
@@ -427,10 +427,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.6401508916323732</v>
+        <v>0.3869142857142857</v>
       </c>
       <c r="D4">
-        <v>2.548677130963522E-07</v>
+        <v>1.716557997522749E-06</v>
       </c>
     </row>
     <row r="5">
@@ -445,10 +445,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.6113991769547326</v>
+        <v>0.3799673469387755</v>
       </c>
       <c r="D5">
-        <v>4.810112946444046E-05</v>
+        <v>3.234267975195473E-07</v>
       </c>
     </row>
     <row r="6">
@@ -463,10 +463,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.6800274348422497</v>
+        <v>0.3206775510204082</v>
       </c>
       <c r="D6">
-        <v>1.305996581422433E-11</v>
+        <v>1.429894972415768E-15</v>
       </c>
     </row>
     <row r="7">
@@ -481,10 +481,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.6381344307270234</v>
+        <v>0.292669387755102</v>
       </c>
       <c r="D7">
-        <v>3.699710962600703E-07</v>
+        <v>2.796328581440632E-21</v>
       </c>
     </row>
   </sheetData>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.4810587174448395</v>
+        <v>0.5127123623584123</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.3463673747100529</v>
+        <v>0.4407668662231769</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.339228267022784</v>
+        <v>0.3467850703613701</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -585,10 +585,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.1578902230355661</v>
+        <v>0.3345758759930962</v>
       </c>
       <c r="D5">
-        <v>7.818528047209838E-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.3730429444426802</v>
+        <v>0.4617923319911552</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.3461900416026312</v>
+        <v>0.4242145571475958</v>
       </c>
       <c r="D7">
         <v>0</v>

</xml_diff>

<commit_message>
sync update spEDM 1.8
</commit_message>
<xml_diff>
--- a/Case of net primary productivity study/Case of net primary productivity study.xlsx
+++ b/Case of net primary productivity study/Case of net primary productivity study.xlsx
@@ -570,7 +570,7 @@
         <v>0.7143327286488832</v>
       </c>
       <c r="D4">
-        <v>2.465172120603125E-234</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -588,7 +588,7 @@
         <v>0.6559515226195394</v>
       </c>
       <c r="D5">
-        <v>4.110980962179658E-185</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -606,7 +606,7 @@
         <v>0.7672520290787253</v>
       </c>
       <c r="D6">
-        <v>4.427251241059769E-291</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
re-execute case study 3
</commit_message>
<xml_diff>
--- a/Case of net primary productivity study/Case of net primary productivity study.xlsx
+++ b/Case of net primary productivity study/Case of net primary productivity study.xlsx
@@ -10,7 +10,8 @@
     <sheet name="gcmc" sheetId="1" r:id="rId1"/>
     <sheet name="gccm" sheetId="2" r:id="rId2"/>
     <sheet name="pcc" sheetId="3" r:id="rId3"/>
-    <sheet name="gd" sheetId="4" r:id="rId4"/>
+    <sheet name="directlingam" sheetId="4" r:id="rId4"/>
+    <sheet name="gd" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -662,12 +663,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>npp</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>npp</t>
         </is>
       </c>
       <c r="C2">
@@ -680,12 +681,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>npp</t>
+          <t>tem</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>tem</t>
+          <t>npp</t>
         </is>
       </c>
       <c r="C3">
@@ -698,12 +699,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>npp</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>npp</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="C4">
@@ -716,12 +717,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>tem</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tem</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="C5">
@@ -734,12 +735,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tem</t>
+          <t>npp</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>npp</t>
+          <t>tem</t>
         </is>
       </c>
       <c r="C6">
@@ -752,12 +753,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tem</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>tem</t>
         </is>
       </c>
       <c r="C7">
@@ -811,6 +812,146 @@
         </is>
       </c>
       <c r="C2">
+        <v>0.3756260251040425</v>
+      </c>
+      <c r="D2">
+        <v>3.642653099578032E-126</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>tem</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>npp</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>6.553671515938445E-28</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>npp</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pre</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>3.642653099578032E-126</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tem</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>pre</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>2.31191231028444E-93</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>npp</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tem</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>0.003965936370808507</v>
+      </c>
+      <c r="D6">
+        <v>6.553671515938445E-28</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>pre</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tem</t>
+        </is>
+      </c>
+      <c r="C7">
+        <v>0.008164496560567478</v>
+      </c>
+      <c r="D7">
+        <v>2.31191231028444E-93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>cause</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>effect</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>cs</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>sig</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>pre</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>npp</t>
+        </is>
+      </c>
+      <c r="C2">
         <v>0.6654054331056385</v>
       </c>
       <c r="D2">

</xml_diff>